<commit_message>
🖼️ Improve image compression and increase upload limits for Vercel
</commit_message>
<xml_diff>
--- a/public/data/orders.xlsx
+++ b/public/data/orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -414,6 +414,7 @@
     <col min="13" max="13" width="20.83203125" customWidth="1"/>
     <col min="14" max="14" width="20.83203125" customWidth="1"/>
     <col min="15" max="15" width="20.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,9 +517,59 @@
         <v>معلق</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ORD-0033</v>
+      </c>
+      <c r="B3" t="str">
+        <v>February 14, 2026 at 04:34 PM</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Belal Ahmed Mohamed</v>
+      </c>
+      <c r="D3" t="str">
+        <v>01220293561</v>
+      </c>
+      <c r="E3" t="str">
+        <v>nn787897@gmail.com</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Black Honey</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>100</v>
+      </c>
+      <c r="I3">
+        <v>100</v>
+      </c>
+      <c r="J3" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="K3" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="L3" t="str">
+        <v xml:space="preserve">3 شارع الملكه </v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v>بدون ملاحظات</v>
+      </c>
+      <c r="O3" t="str">
+        <v>تحويل بنكي للرقم 01012622315</v>
+      </c>
+      <c r="P3" t="str">
+        <v>معلق</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: remove Paymob integration and simplify to Vodafone Cash only
REMOVED:
- Paymob payment gateway library (lib/paymob.ts)
- All Paymob-related imports and functions (visa, paypal, cashcollection, kiosk)
- Complex payment initiation logic for multiple payment methods

UPDATED:
- payment/initiate route now simplified for Vodafone Cash only
- cart page payment handler refactored to remove Paymob dependencies
- Email service (Brevo) now gracefully handles missing API key without failing order

FIXED:
- Brevo email errors no longer block order submission
- Email notifications fail silently with logging instead of blocking checkout
- Reduced API call complexity from 5 payment methods to 1 (Vodafone Cash)

RATIONALE:
- Removes unnecessary complexity and external dependencies
- Vodafone Cash only uses manual screenshot upload (no payment gateway needed)
- Improves error handling and order flow resilience
</commit_message>
<xml_diff>
--- a/public/data/orders.xlsx
+++ b/public/data/orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P5"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -617,9 +617,59 @@
         <v>معلق</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ORD-0036</v>
+      </c>
+      <c r="B5" t="str">
+        <v>February 15, 2026 at 09:15 PM</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Belal Ahmed Mohamed</v>
+      </c>
+      <c r="D5" t="str">
+        <v>01220293561</v>
+      </c>
+      <c r="E5" t="str">
+        <v>nn787897@gmail.com</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Burgundy</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>100</v>
+      </c>
+      <c r="I5">
+        <v>100</v>
+      </c>
+      <c r="J5" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="K5" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="L5" t="str">
+        <v xml:space="preserve">3 شارع الملكه </v>
+      </c>
+      <c r="M5" t="str">
+        <v>كليه الزراعه</v>
+      </c>
+      <c r="N5" t="str">
+        <v>بدون ملاحظات</v>
+      </c>
+      <c r="O5" t="str">
+        <v>تحويل بنكي للرقم 01012622315</v>
+      </c>
+      <c r="P5" t="str">
+        <v>معلق</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
debug: add Brevo API key diagnostics
</commit_message>
<xml_diff>
--- a/public/data/orders.xlsx
+++ b/public/data/orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P6"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -667,9 +667,59 @@
         <v>معلق</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ORD-0037</v>
+      </c>
+      <c r="B6" t="str">
+        <v>February 15, 2026 at 09:37 PM</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Belal Ahmed Mohamed</v>
+      </c>
+      <c r="D6" t="str">
+        <v>01220293561</v>
+      </c>
+      <c r="E6" t="str">
+        <v>nn787897@gmail.com</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Black Honey</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>100</v>
+      </c>
+      <c r="I6">
+        <v>100</v>
+      </c>
+      <c r="J6" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="K6" t="str">
+        <v>shobra</v>
+      </c>
+      <c r="L6" t="str">
+        <v xml:space="preserve">3 شارع الملكه </v>
+      </c>
+      <c r="M6" t="str">
+        <v>كليه الزراعه</v>
+      </c>
+      <c r="N6" t="str">
+        <v>بدون ملاحظات</v>
+      </c>
+      <c r="O6" t="str">
+        <v>تحويل بنكي للرقم 01012622315</v>
+      </c>
+      <c r="P6" t="str">
+        <v>معلق</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
clean: remove debug logs from Brevo email service
</commit_message>
<xml_diff>
--- a/public/data/orders.xlsx
+++ b/public/data/orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P7"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -717,9 +717,59 @@
         <v>معلق</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ORD-0038</v>
+      </c>
+      <c r="B7" t="str">
+        <v>February 15, 2026 at 09:48 PM</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Belal Ahmed Mohamed</v>
+      </c>
+      <c r="D7" t="str">
+        <v>01220293561</v>
+      </c>
+      <c r="E7" t="str">
+        <v>nn787897@gmail.com</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Black Honey</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>100</v>
+      </c>
+      <c r="I7">
+        <v>100</v>
+      </c>
+      <c r="J7" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="K7" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="L7" t="str">
+        <v xml:space="preserve">3 شارع الملكه </v>
+      </c>
+      <c r="M7" t="str">
+        <v>كليه الزراعه</v>
+      </c>
+      <c r="N7" t="str">
+        <v>بدون ملاحظات</v>
+      </c>
+      <c r="O7" t="str">
+        <v>تحويل بنكي للرقم 01012622315</v>
+      </c>
+      <c r="P7" t="str">
+        <v>معلق</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: mobile order flow, Brevo, Telegram, image upload, and thank you page (mobile parity)
</commit_message>
<xml_diff>
--- a/public/data/orders.xlsx
+++ b/public/data/orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P8"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -767,9 +767,59 @@
         <v>معلق</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ORD-0042</v>
+      </c>
+      <c r="B8" t="str">
+        <v>February 16, 2026 at 11:37 AM</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Belal Ahmed Mohamed</v>
+      </c>
+      <c r="D8" t="str">
+        <v>01220293561</v>
+      </c>
+      <c r="E8" t="str">
+        <v>nn787897@gmail.com</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Black Honey</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>100</v>
+      </c>
+      <c r="I8">
+        <v>100</v>
+      </c>
+      <c r="J8" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="K8" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="L8" t="str">
+        <v xml:space="preserve">3 شارع الملكه </v>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v>بدون ملاحظات</v>
+      </c>
+      <c r="O8" t="str">
+        <v>تحويل بنكي للرقم 01012622315</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: Telegram photo upload using Web FormData/Blob, Brevo key cleaning
- Replace form-data npm package with native Web API FormData + Blob for Telegram photo uploads
- This fixes 'Unexpected end of JSON input' error (form-data streams incompatible with fetch)
- Add response.text() + safe JSON.parse to handle non-JSON Telegram responses
- Clean Brevo API key: strip quotes, newlines, whitespace (fixes 'Key not found')
- Add detailed Brevo key diagnostics (length, prefix, suffix)
- Fix sendTelegram route: use sendPhotoToTelegram directly (avoid duplicate message)
- Add transferImageMime to sendTelegram TelegramPayload interface
</commit_message>
<xml_diff>
--- a/public/data/orders.xlsx
+++ b/public/data/orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P11"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -817,9 +817,159 @@
         <v>Pending</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ORD-0043</v>
+      </c>
+      <c r="B9" t="str">
+        <v>February 16, 2026 at 12:42 PM</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Lingo</v>
+      </c>
+      <c r="D9" t="str">
+        <v>01220293561</v>
+      </c>
+      <c r="E9" t="str">
+        <v>nn787897@gmail.com</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Wine</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>100</v>
+      </c>
+      <c r="I9">
+        <v>100</v>
+      </c>
+      <c r="J9" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="K9" t="str">
+        <v>shobra</v>
+      </c>
+      <c r="L9" t="str">
+        <v xml:space="preserve">3 شارع الملكه </v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v>بدون ملاحظات</v>
+      </c>
+      <c r="O9" t="str">
+        <v>تحويل بنكي للرقم 01012622315</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ORD-0044</v>
+      </c>
+      <c r="B10" t="str">
+        <v>February 16, 2026 at 12:46 PM</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Belal Ahmed Mohamed</v>
+      </c>
+      <c r="D10" t="str">
+        <v>01220293561</v>
+      </c>
+      <c r="E10" t="str">
+        <v>nn787897@gmail.com</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Wine</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>100</v>
+      </c>
+      <c r="I10">
+        <v>100</v>
+      </c>
+      <c r="J10" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="K10" t="str">
+        <v>shobra</v>
+      </c>
+      <c r="L10" t="str">
+        <v xml:space="preserve">3 شارع الملكه </v>
+      </c>
+      <c r="M10" t="str">
+        <v>كليه الزراعه</v>
+      </c>
+      <c r="N10" t="str">
+        <v>call me</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Vodafone Cash</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ORD-0044</v>
+      </c>
+      <c r="B11" t="str">
+        <v>February 16, 2026 at 12:46 PM</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Belal Ahmed Mohamed</v>
+      </c>
+      <c r="D11" t="str">
+        <v>01220293561</v>
+      </c>
+      <c r="E11" t="str">
+        <v>nn787897@gmail.com</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Mocha</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>100</v>
+      </c>
+      <c r="I11">
+        <v>100</v>
+      </c>
+      <c r="J11" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="K11" t="str">
+        <v>shobra</v>
+      </c>
+      <c r="L11" t="str">
+        <v xml:space="preserve">3 شارع الملكه </v>
+      </c>
+      <c r="M11" t="str">
+        <v>كليه الزراعه</v>
+      </c>
+      <c r="N11" t="str">
+        <v>call me</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Vodafone Cash</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add brevo-test API route
</commit_message>
<xml_diff>
--- a/public/data/orders.xlsx
+++ b/public/data/orders.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P12"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -967,9 +967,59 @@
         <v>Pending</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ORD-0045</v>
+      </c>
+      <c r="B12" t="str">
+        <v>February 16, 2026 at 12:51 PM</v>
+      </c>
+      <c r="C12" t="str">
+        <v>belal</v>
+      </c>
+      <c r="D12" t="str">
+        <v>012 20293561</v>
+      </c>
+      <c r="E12" t="str">
+        <v>bollaahmed85@gmail.com</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Lip Balm</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>100</v>
+      </c>
+      <c r="I12">
+        <v>100</v>
+      </c>
+      <c r="J12" t="str">
+        <v>cairo</v>
+      </c>
+      <c r="K12" t="str">
+        <v>shobra</v>
+      </c>
+      <c r="L12" t="str">
+        <v xml:space="preserve">3 شارع الملكه </v>
+      </c>
+      <c r="M12" t="str">
+        <v>كليه الزراعه</v>
+      </c>
+      <c r="N12" t="str">
+        <v>شسيبلاتنمكط</v>
+      </c>
+      <c r="O12" t="str">
+        <v>تحويل بنكي للرقم 01012622315</v>
+      </c>
+      <c r="P12" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>